<commit_message>
Update conversion and indicator export logic + Excel spec
</commit_message>
<xml_diff>
--- a/data/examples/S1CRU1_AnalysisTable_Specification.xlsx
+++ b/data/examples/S1CRU1_AnalysisTable_Specification.xlsx
@@ -1,15 +1,40 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <workbookPr defaultThemeVersion="202300"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://regtechnet-my.sharepoint.com/personal/ce-raphael_colin_regnology_net/Documents/Bureau/github/excel-to-indicator-mcp/data/examples/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_8587D4973538C0C3A16C10FF0C9CC65889149073" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
     <sheet name="#TEMPLATE" sheetId="1" r:id="rId1"/>
     <sheet name="Data" sheetId="2" r:id="rId2"/>
   </sheets>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="58">
   <si>
     <t>#CELL</t>
   </si>
@@ -189,15 +214,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
-    <numFmt numFmtId="164" formatCode="#,##0"/>
-    <numFmt numFmtId="165" formatCode="#,##0.00"/>
-    <numFmt numFmtId="166" formatCode="0"/>
-    <numFmt numFmtId="167" formatCode="0.00%"/>
-    <numFmt numFmtId="168" formatCode="@"/>
-  </numFmts>
-  <fonts count="6">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -352,127 +370,460 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0"/>
-    <xf xfId="0" fontId="1" applyFont="1" numFmtId="0" fillId="0" borderId="0" applyBorder="1" applyAlignment="1">
+  <cellXfs count="36">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf xfId="0" fontId="1" applyFont="1" numFmtId="0" fillId="0" borderId="0" applyBorder="1"/>
-    <xf xfId="0" fontId="2" applyFont="1" numFmtId="0" fillId="0" borderId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf xfId="0" fontId="2" applyFont="1" numFmtId="0" fillId="0" borderId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf xfId="0" fontId="2" applyFont="1" numFmtId="0" fillId="0" borderId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf xfId="0" fontId="2" applyFont="1" numFmtId="0" fillId="0" borderId="2" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf xfId="0" fontId="2" applyFont="1" numFmtId="0" fillId="0" borderId="3" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf xfId="0" fontId="2" applyFont="1" numFmtId="0" fillId="0" borderId="3" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf xfId="0" fontId="2" applyFont="1" numFmtId="0" fillId="2" applyFill="1" borderId="2" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf xfId="0" fontId="2" applyFont="1" numFmtId="0" fillId="2" applyFill="1" borderId="2" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" fontId="2" applyFont="1" numFmtId="164" applyNumberFormat="1" fillId="0" borderId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf xfId="0" fontId="2" applyFont="1" numFmtId="164" applyNumberFormat="1" fillId="0" borderId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf xfId="0" fontId="2" applyFont="1" numFmtId="164" applyNumberFormat="1" fillId="0" borderId="3" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf xfId="0" fontId="2" applyFont="1" numFmtId="164" applyNumberFormat="1" fillId="0" borderId="3" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf xfId="0" fontId="2" applyFont="1" numFmtId="165" applyNumberFormat="1" fillId="0" borderId="3" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="4" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf xfId="0" fontId="2" applyFont="1" numFmtId="166" applyNumberFormat="1" fillId="3" applyFill="1" borderId="2" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" fontId="2" applyFont="1" numFmtId="167" applyNumberFormat="1" fillId="0" borderId="2" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf xfId="0" fontId="2" applyFont="1" numFmtId="168" applyNumberFormat="1" fillId="0" borderId="3" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf xfId="0" fontId="3" applyFont="1" numFmtId="0" fillId="0" borderId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf xfId="0" fontId="3" applyFont="1" numFmtId="0" fillId="0" borderId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf xfId="0" fontId="4" applyFont="1" numFmtId="0" fillId="4" applyFill="1" borderId="4" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" fontId="4" applyFont="1" numFmtId="0" fillId="4" applyFill="1" borderId="5" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" fontId="4" applyFont="1" numFmtId="0" fillId="4" applyFill="1" borderId="2" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" fontId="4" applyFont="1" numFmtId="166" applyNumberFormat="1" fillId="0" borderId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" fontId="4" applyFont="1" numFmtId="166" applyNumberFormat="1" fillId="4" applyFill="1" borderId="4" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="4" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" fontId="4" applyFont="1" numFmtId="166" applyNumberFormat="1" fillId="4" applyFill="1" borderId="2" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="4" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" fontId="4" applyFont="1" numFmtId="166" applyNumberFormat="1" fillId="4" applyFill="1" borderId="3" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="4" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" fontId="4" applyFont="1" numFmtId="168" applyNumberFormat="1" fillId="4" applyFill="1" borderId="4" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" fontId="5" applyFont="1" numFmtId="0" fillId="5" applyFill="1" borderId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf xfId="0" fontId="5" applyFont="1" numFmtId="0" fillId="6" applyFill="1" borderId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf xfId="0" fontId="5" applyFont="1" numFmtId="0" fillId="7" applyFill="1" borderId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf xfId="0" fontId="5" applyFont="1" numFmtId="0" fillId="8" applyFill="1" borderId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf xfId="0" fontId="5" applyFont="1" numFmtId="0" fillId="9" applyFill="1" borderId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="0E2841"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="E8E8E8"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="156082"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="E97132"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="196B24"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="0F9ED5"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="A02B93"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="4EA72E"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="467886"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="96607D"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+                <a:tint val="67000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+                <a:tint val="73000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+                <a:tint val="81000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:satMod val="103000"/>
+                <a:lumMod val="102000"/>
+                <a:tint val="94000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:satMod val="110000"/>
+                <a:lumMod val="100000"/>
+                <a:shade val="100000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+                <a:shade val="78000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="63000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:tint val="95000"/>
+            <a:satMod val="170000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="93000"/>
+                <a:satMod val="150000"/>
+                <a:shade val="98000"/>
+                <a:lumMod val="102000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:tint val="98000"/>
+                <a:satMod val="130000"/>
+                <a:shade val="90000"/>
+                <a:lumMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="63000"/>
+                <a:satMod val="120000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
+  <a:extraClrSchemeLst/>
+  <a:extLst>
+    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+    </a:ext>
+  </a:extLst>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:B4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="13.6412" customWidth="1"/>
-    <col min="2" max="2" width="13.6412" customWidth="1"/>
+    <col min="1" max="2" width="13.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B1" s="29" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" s="29" t="s">
         <v>7</v>
       </c>
@@ -480,7 +831,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="29" t="s">
         <v>1</v>
       </c>
@@ -488,7 +839,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="29" t="s">
         <v>4</v>
       </c>
@@ -497,38 +848,27 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:Q16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" outlineLevelCol="1" outlineLevelRow="1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" outlineLevelRow="1" outlineLevelCol="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" outlineLevel="1" width="13.6412" customWidth="1"/>
-    <col min="2" max="2" outlineLevel="1" width="13.6412" customWidth="1"/>
-    <col min="3" max="3" outlineLevel="1" width="13.6412" customWidth="1"/>
-    <col min="4" max="4" width="10.9872" customWidth="1"/>
-    <col min="5" max="5" width="23.843" customWidth="1"/>
-    <col min="6" max="6" width="23.843" customWidth="1"/>
-    <col min="7" max="7" width="23.843" customWidth="1"/>
-    <col min="8" max="8" width="23.843" customWidth="1"/>
-    <col min="9" max="9" width="23.843" customWidth="1"/>
-    <col min="10" max="10" width="23.843" customWidth="1"/>
-    <col min="11" max="11" width="23.843" customWidth="1"/>
-    <col min="12" max="12" width="23.843" customWidth="1"/>
-    <col min="13" max="13" width="23.843" customWidth="1"/>
-    <col min="14" max="14" width="23.843" customWidth="1"/>
-    <col min="15" max="15" width="23.843" customWidth="1"/>
-    <col min="16" max="16" width="10.9872" customWidth="1"/>
-    <col min="17" max="17" width="14.2052" customWidth="1"/>
+    <col min="1" max="3" width="13.5703125" customWidth="1" outlineLevel="1"/>
+    <col min="4" max="4" width="11" customWidth="1"/>
+    <col min="5" max="15" width="23.85546875" customWidth="1"/>
+    <col min="16" max="16" width="11" customWidth="1"/>
+    <col min="17" max="17" width="14.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" outlineLevel="1">
+    <row r="1" spans="1:17" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B1" s="32" t="s">
         <v>6</v>
       </c>
@@ -572,7 +912,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" outlineLevel="1">
+    <row r="2" spans="1:17" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A2" s="32" t="s">
         <v>6</v>
       </c>
@@ -593,7 +933,7 @@
       <c r="P2" s="3"/>
       <c r="Q2" s="1"/>
     </row>
-    <row r="3" outlineLevel="1">
+    <row r="3" spans="1:17" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A3" s="31" t="s">
         <v>2</v>
       </c>
@@ -614,7 +954,7 @@
       <c r="P3" s="3"/>
       <c r="Q3" s="1"/>
     </row>
-    <row r="4" ht="14" customHeight="1">
+    <row r="4" spans="1:17" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="29" t="s">
         <v>3</v>
       </c>
@@ -635,7 +975,7 @@
       <c r="P4" s="3"/>
       <c r="Q4" s="1"/>
     </row>
-    <row r="5" ht="14" customHeight="1">
+    <row r="5" spans="1:17" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="29" t="s">
         <v>3</v>
       </c>
@@ -656,17 +996,17 @@
       <c r="P5" s="3"/>
       <c r="Q5" s="1"/>
     </row>
-    <row r="6" ht="14" customHeight="1">
+    <row r="6" spans="1:17" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="29" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
-      <c r="E6" s="19" t="s">
+      <c r="E6" s="34" t="s">
         <v>53</v>
       </c>
-      <c r="F6" s="3"/>
+      <c r="F6" s="35"/>
       <c r="G6" s="3"/>
       <c r="H6" s="20" t="s">
         <v>9</v>
@@ -691,7 +1031,7 @@
       </c>
       <c r="Q6" s="1"/>
     </row>
-    <row r="7" outlineLevel="1">
+    <row r="7" spans="1:17" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A7" s="33" t="s">
         <v>0</v>
       </c>
@@ -714,7 +1054,7 @@
       <c r="P7" s="3"/>
       <c r="Q7" s="1"/>
     </row>
-    <row r="8" ht="25" customHeight="1">
+    <row r="8" spans="1:17" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="29" t="s">
         <v>3</v>
       </c>
@@ -739,7 +1079,7 @@
       <c r="P8" s="3"/>
       <c r="Q8" s="1"/>
     </row>
-    <row r="9" outlineLevel="1">
+    <row r="9" spans="1:17" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A9" s="33" t="s">
         <v>0</v>
       </c>
@@ -762,7 +1102,7 @@
       <c r="P9" s="3"/>
       <c r="Q9" s="1"/>
     </row>
-    <row r="10" ht="25" customHeight="1">
+    <row r="10" spans="1:17" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="29" t="s">
         <v>3</v>
       </c>
@@ -787,7 +1127,7 @@
       <c r="P10" s="3"/>
       <c r="Q10" s="1"/>
     </row>
-    <row r="11" outlineLevel="1">
+    <row r="11" spans="1:17" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A11" s="33" t="s">
         <v>0</v>
       </c>
@@ -812,7 +1152,7 @@
       <c r="P11" s="3"/>
       <c r="Q11" s="1"/>
     </row>
-    <row r="12" ht="14" customHeight="1">
+    <row r="12" spans="1:17" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="29" t="s">
         <v>3</v>
       </c>
@@ -833,7 +1173,7 @@
       <c r="P12" s="3"/>
       <c r="Q12" s="1"/>
     </row>
-    <row r="13" ht="38" customHeight="1">
+    <row r="13" spans="1:17" ht="38.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="29" t="s">
         <v>3</v>
       </c>
@@ -876,7 +1216,7 @@
       <c r="P13" s="3"/>
       <c r="Q13" s="1"/>
     </row>
-    <row r="14" ht="14" customHeight="1">
+    <row r="14" spans="1:17" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="29" t="s">
         <v>3</v>
       </c>
@@ -919,7 +1259,7 @@
       <c r="P14" s="3"/>
       <c r="Q14" s="1"/>
     </row>
-    <row r="15" ht="14" customHeight="1">
+    <row r="15" spans="1:17" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="3"/>
       <c r="C15" s="30" t="s">
         <v>12</v>
@@ -939,7 +1279,7 @@
       <c r="P15" s="3"/>
       <c r="Q15" s="1"/>
     </row>
-    <row r="16" outlineLevel="1">
+    <row r="16" spans="1:17" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A16" s="33" t="s">
         <v>0</v>
       </c>
@@ -984,6 +1324,7 @@
   <mergeCells count="1">
     <mergeCell ref="E6:F6"/>
   </mergeCells>
-  <pageSetup orientation="portrait"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>